<commit_message>
READ ME FIRST: full readiness explainer - 5 components in plain English + score-level ladder (<30 resting / 40-60 mixed / 70+ coiled) + 8/1 calibration honesty (no separation, catalyst-blind, works neither as green light nor veto)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/universe_2026-07-31.xlsx
+++ b/reports/universe_2026-07-31.xlsx
@@ -1775,7 +1775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B66"/>
+  <dimension ref="A1:B67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1826,7 +1826,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>2026-08-01 16:01 local</t>
+          <t>2026-08-01 16:09 local</t>
         </is>
       </c>
     </row>
@@ -2314,77 +2314,89 @@
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>Readiness 0-100 = poised-to-move (UNCALIBRATED - ranks, does not veto). The gates answer 'is it SAFE to buy'; this answers 'does it MOVE soon'. Five checks worth 20 points each: bands coiled tight, price within reach of its trigger (the 20-day high), volume flowing in, momentum turning up, beating the market. HOW TO READ IT: 60+ = the spring is loading. Below 40 = expect sideways first - DGX read 26/100 the night it topped the gate list on trend strength (ADX 42) and then went nowhere, exactly as scored (the 7/31 post-mortem that created this column). The text after the number names the strongest or weakest ingredients. It RANKS which candidate to look at first; it never blocks a trade on its own until the Friday reviews prove it deserves that power. 'n/a' = the overnight scoring step did not run for that name.</t>
+          <t>Poised-to-move score. The gates answer 'is it SAFE to buy'; this answers 'is a move LOADING soon, in the trade's direction'. Five classic ready-to-run checks, 20 points each: (1) SQUEEZE - price bands coiled to their tightest in months = energy stored, the closest thing to a true 'ready' signal; (2) TRIGGER - how close price sits to its 20-day high, i.e. how short the fuse is (one good day vs a long grind); (3) VOLUME - quiet accumulation: big money sneaking in while price goes sideways; (4) MOMENTUM - the turn before the turn: momentum just changed direction toward the trade; (5) RELATIVE STRENGTH - beating the market at a 60-day extreme, money singling this name out right now. The text after the number names the lit and dead ingredients - READ THE TEXT, not just the number: a 54 built on 'tight coil + volume' is a different animal from a 54 built on 'strong but bands blown out'. 'n/a' = the overnight scoring step did not run for that name.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>Magical (CCI-20)</t>
+          <t>Readiness - the levels</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>Above +100 = overbought, below -100 = oversold. NOTE: measured 2026-07-22 across 1,725 signals, this cut does NOT separate returns (0.03pt over 21 days). Treat as context, not a veto.</t>
+          <t>UNDER ~30 = RESTING: energy already spent (bands wide after a move) or nothing loading - expect sideways unless news does the work; a fine HOLDING can score here (DGX read 26 and beat the market that week while going nowhere vs its entry). 40-60 = MIXED: two or three parts lit - the driver text decides whether it's interesting. 70+ = RARE/COILED: most parts firing together; CORT hit 95 on 7/7 and ran +22%. PRIME SETUP tag (options tab) = tight squeeze + cheap premium at once - the one pattern with real published history. NOW THE HONEST PART (first calibration look, 2026-08-01): comparing the big skipped runners vs skipped picks that went NOWHERE, pick-day scores showed NO separation (means 47 vs 43) - PSA scored 80 and never moved 2%; CAKE scored 16 and ran +30% on earnings. The score sees STORED ENERGY only - it is blind to catalyst movers (news, earnings gaps) and says nothing about direction or exact timing. So it works BOTH ways: a high score is NOT a green light and a low score is NOT a veto. Use it to decide which gate-passer to LOOK AT first and what posture you're buying (coiled vs resting), never as the reason to trade. The nightly scan is collecting the forward evidence; Friday reviews decide if any threshold ever earns real power.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>ZLSMA-50</t>
+          <t>Magical (CCI-20)</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>The trend line. Price below it on a buy signal is a structural fail.</t>
+          <t>Above +100 = overbought, below -100 = oversold. NOTE: measured 2026-07-22 across 1,725 signals, this cut does NOT separate returns (0.03pt over 21 days). Treat as context, not a veto.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>Chandelier Exit</t>
+          <t>ZLSMA-50</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>Flips BUY/SELL. The label price is the STOP level, not an entry.</t>
+          <t>The trend line. Price below it on a buy signal is a structural fail.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>Regime PASS</t>
+          <t>Chandelier Exit</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>Above a rising 200-day and beating SPY -&gt; normal size.</t>
+          <t>Flips BUY/SELL. The label price is the STOP level, not an entry.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
+          <t>Regime PASS</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>Above a rising 200-day and beating SPY -&gt; normal size.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
           <t>Regime REPAIR</t>
         </is>
       </c>
-      <c r="B65" s="6" t="inlineStr">
+      <c r="B66" s="6" t="inlineStr">
         <is>
           <t>Below the 200-day -&gt; starter size only.</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="7" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="7" t="inlineStr">
         <is>
           <t>Regime DEEP-FAIL</t>
         </is>
       </c>
-      <c r="B66" s="8" t="inlineStr">
+      <c r="B67" s="8" t="inlineStr">
         <is>
           <t>More than 10% below the 200-day -&gt; watch only, no size.</t>
         </is>
@@ -30747,7 +30759,7 @@
       </c>
       <c r="B4" s="17" t="inlineStr">
         <is>
-          <t>2026-08-01 16:01 local</t>
+          <t>2026-08-01 16:09 local</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
RESTED LEADER tag (display-only rename of rest-continuation cohort, Omar 8/1): column on Fresh Buys + Gated Longs with on-trial label + zero-weight tooltip; preregistration addendum (rule untouched); MLI+HQY tagged in rebuilt 7/31 workbook
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/universe_2026-07-31.xlsx
+++ b/reports/universe_2026-07-31.xlsx
@@ -23,8 +23,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 - Run Summary" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2 - Fresh Buys'!$A$1:$AA$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'2b - Gated Longs'!$A$1:$N$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2 - Fresh Buys'!$A$1:$AB$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'2b - Gated Longs'!$A$1:$O$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'3 - Plans'!$A$1:$K$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'4 - Blocked'!$A$1:$K$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'5 - Sell Mode'!$A$1:$M$1</definedName>
@@ -964,11 +964,17 @@
     </comment>
     <comment ref="Z1" authorId="0" shapeId="0">
       <text>
+        <t>RESTED LEADER = this name fits the pre-registered second-leg profile tonight: proven trend (ADX 25+), buyers firmly in control (DI margin 10+), RESTING (readiness &lt;=30) on quiet volume (RVOL &lt;1.2). July's +15% winners were overwhelmingly this shape - NOT coiled squeezes. ON TRIAL (an experiment, verdict 2026-09-25): the tag carries ZERO weight in gates, sizing or ranking until the forward test proves it. Blank = does not fit the profile tonight - not a defect.
+(Full guide: 'READ ME FIRST' tab)</t>
+      </text>
+    </comment>
+    <comment ref="AA1" authorId="0" shapeId="0">
+      <text>
         <t>Next scheduled catalyst for this name - earnings within 7 days, or a Phase-3 trial readout window. Blank = none flagged. From build_catalyst_calendar.py.
 (Full guide: 'READ ME FIRST' tab)</t>
       </text>
     </comment>
-    <comment ref="AA1" authorId="0" shapeId="0">
+    <comment ref="AB1" authorId="0" shapeId="0">
       <text>
         <t>What the catalyst is and the suggested ACTION. Earnings: trim into the print, re-enter post-print only if it beats AND holds (PEAD). Biopharma: BINARY - defined-risk / awareness only, never hold a momentum long through it.
 (Full guide: 'READ ME FIRST' tab)</t>
@@ -1058,11 +1064,17 @@
     </comment>
     <comment ref="M1" authorId="0" shapeId="0">
       <text>
+        <t>RESTED LEADER = this name fits the pre-registered second-leg profile tonight: proven trend (ADX 25+), buyers firmly in control (DI margin 10+), RESTING (readiness &lt;=30) on quiet volume (RVOL &lt;1.2). July's +15% winners were overwhelmingly this shape - NOT coiled squeezes. ON TRIAL (an experiment, verdict 2026-09-25): the tag carries ZERO weight in gates, sizing or ranking until the forward test proves it. Blank = does not fit the profile tonight - not a defect.
+(Full guide: 'READ ME FIRST' tab)</t>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0" shapeId="0">
+      <text>
         <t>Next scheduled catalyst for this name - earnings within 7 days, or a Phase-3 trial readout window. Blank = none flagged. From build_catalyst_calendar.py.
 (Full guide: 'READ ME FIRST' tab)</t>
       </text>
     </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
+    <comment ref="O1" authorId="0" shapeId="0">
       <text>
         <t>What the catalyst is and the suggested ACTION. Earnings: trim into the print, re-enter post-print only if it beats AND holds (PEAD). Biopharma: BINARY - defined-risk / awareness only, never hold a momentum long through it.
 (Full guide: 'READ ME FIRST' tab)</t>
@@ -1826,7 +1838,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>2026-08-01 16:09 local</t>
+          <t>2026-08-01 17:32 local</t>
         </is>
       </c>
     </row>
@@ -30759,7 +30771,7 @@
       </c>
       <c r="B4" s="17" t="inlineStr">
         <is>
-          <t>2026-08-01 16:09 local</t>
+          <t>2026-08-01 17:32 local</t>
         </is>
       </c>
     </row>
@@ -32760,7 +32772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA79"/>
+  <dimension ref="A1:AB79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -32788,8 +32800,9 @@
     <col width="12" customWidth="1" min="23" max="23"/>
     <col width="26" customWidth="1" min="24" max="24"/>
     <col width="55" customWidth="1" min="25" max="25"/>
-    <col width="22" customWidth="1" min="26" max="26"/>
-    <col width="62" customWidth="1" min="27" max="27"/>
+    <col width="20" customWidth="1" min="26" max="26"/>
+    <col width="22" customWidth="1" min="27" max="27"/>
+    <col width="62" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -32920,10 +32933,15 @@
       </c>
       <c r="Z1" s="12" t="inlineStr">
         <is>
+          <t>Rested Leader</t>
+        </is>
+      </c>
+      <c r="AA1" s="12" t="inlineStr">
+        <is>
           <t>Catalyst</t>
         </is>
       </c>
-      <c r="AA1" s="12" t="inlineStr">
+      <c r="AB1" s="12" t="inlineStr">
         <is>
           <t>Catalyst View</t>
         </is>
@@ -33025,8 +33043,9 @@
           <t>Passes every gate: regime, trend strength (ADX)&gt;=20, +DI&gt;-DI, above its trend line (ZLSMA), and liquid enough for a $85,000 position.</t>
         </is>
       </c>
-      <c r="Z2" s="19" t="inlineStr"/>
+      <c r="Z2" s="19" t="n"/>
       <c r="AA2" s="19" t="inlineStr"/>
+      <c r="AB2" s="19" t="inlineStr"/>
     </row>
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="17" t="n">
@@ -33124,8 +33143,9 @@
           <t>Passes every gate: regime, trend strength (ADX)&gt;=20, +DI&gt;-DI, above its trend line (ZLSMA), and liquid enough for a $85,000 position.</t>
         </is>
       </c>
-      <c r="Z3" s="19" t="inlineStr"/>
+      <c r="Z3" s="19" t="n"/>
       <c r="AA3" s="19" t="inlineStr"/>
+      <c r="AB3" s="19" t="inlineStr"/>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="17" t="n">
@@ -33223,8 +33243,9 @@
           <t>regime REPAIR (23.0346% vs the 200-day average) - starter size only</t>
         </is>
       </c>
-      <c r="Z4" s="19" t="inlineStr"/>
+      <c r="Z4" s="19" t="n"/>
       <c r="AA4" s="19" t="inlineStr"/>
+      <c r="AB4" s="19" t="inlineStr"/>
     </row>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="17" t="n">
@@ -33322,8 +33343,9 @@
           <t>Passes every gate: regime, trend strength (ADX)&gt;=20, +DI&gt;-DI, above its trend line (ZLSMA), and liquid enough for a $85,000 position.</t>
         </is>
       </c>
-      <c r="Z5" s="19" t="inlineStr"/>
+      <c r="Z5" s="19" t="n"/>
       <c r="AA5" s="19" t="inlineStr"/>
+      <c r="AB5" s="19" t="inlineStr"/>
     </row>
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="17" t="n">
@@ -33415,8 +33437,9 @@
           <t>regime REPAIR (8.4497% vs the 200-day average) - starter size only</t>
         </is>
       </c>
-      <c r="Z6" s="19" t="inlineStr"/>
+      <c r="Z6" s="19" t="n"/>
       <c r="AA6" s="19" t="inlineStr"/>
+      <c r="AB6" s="19" t="inlineStr"/>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="17" t="n">
@@ -33508,8 +33531,9 @@
           <t>Passes every gate: regime, trend strength (ADX)&gt;=20, +DI&gt;-DI, above its trend line (ZLSMA), and liquid enough for a $85,000 position.</t>
         </is>
       </c>
-      <c r="Z7" s="19" t="inlineStr"/>
+      <c r="Z7" s="19" t="n"/>
       <c r="AA7" s="19" t="inlineStr"/>
+      <c r="AB7" s="19" t="inlineStr"/>
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="17" t="n">
@@ -33607,8 +33631,9 @@
           <t>Passes every gate: regime, trend strength (ADX)&gt;=20, +DI&gt;-DI, above its trend line (ZLSMA), and liquid enough for a $85,000 position.</t>
         </is>
       </c>
-      <c r="Z8" s="19" t="inlineStr"/>
+      <c r="Z8" s="19" t="n"/>
       <c r="AA8" s="19" t="inlineStr"/>
+      <c r="AB8" s="19" t="inlineStr"/>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="17" t="n">
@@ -33700,8 +33725,9 @@
           <t>regime REPAIR (11.8104% vs the 200-day average) - starter size only</t>
         </is>
       </c>
-      <c r="Z9" s="19" t="inlineStr"/>
+      <c r="Z9" s="19" t="n"/>
       <c r="AA9" s="19" t="inlineStr"/>
+      <c r="AB9" s="19" t="inlineStr"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="23" t="n">
@@ -33799,8 +33825,9 @@
           <t>stop is 14.5% away - volatility cap 12%: a name this wild shrinks a fixed-risk position to a token</t>
         </is>
       </c>
-      <c r="Z10" s="25" t="inlineStr"/>
+      <c r="Z10" s="25" t="n"/>
       <c r="AA10" s="25" t="inlineStr"/>
+      <c r="AB10" s="25" t="inlineStr"/>
     </row>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="23" t="n">
@@ -33892,8 +33919,9 @@
           <t>stop is 5.81x ATR (multiples of a normal day's swing) - so wide the position shrinks to a token (ceiling 4.0x); stop is 17.5% away - volatility...</t>
         </is>
       </c>
-      <c r="Z11" s="25" t="inlineStr"/>
+      <c r="Z11" s="25" t="n"/>
       <c r="AA11" s="25" t="inlineStr"/>
+      <c r="AB11" s="25" t="inlineStr"/>
     </row>
     <row r="12" ht="45" customHeight="1">
       <c r="A12" s="23" t="n">
@@ -33985,8 +34013,9 @@
           <t>-DI 22.0013 &gt;= +DI 20.7429 - sellers in control; stop is 4.70x ATR (multiples of a normal day's swing) - so wide the position shrinks to a toke...</t>
         </is>
       </c>
-      <c r="Z12" s="25" t="inlineStr"/>
+      <c r="Z12" s="25" t="n"/>
       <c r="AA12" s="25" t="inlineStr"/>
+      <c r="AB12" s="25" t="inlineStr"/>
     </row>
     <row r="13" ht="45" customHeight="1">
       <c r="A13" s="23" t="n">
@@ -34084,8 +34113,9 @@
           <t>stop is 4.92x ATR (multiples of a normal day's swing) - so wide the position shrinks to a token (ceiling 4.0x); stop is 31.8% away - volatility...</t>
         </is>
       </c>
-      <c r="Z13" s="25" t="inlineStr"/>
+      <c r="Z13" s="25" t="n"/>
       <c r="AA13" s="25" t="inlineStr"/>
+      <c r="AB13" s="25" t="inlineStr"/>
     </row>
     <row r="14" ht="45" customHeight="1">
       <c r="A14" s="23" t="n">
@@ -34177,8 +34207,9 @@
           <t>stop is 15.1% away - volatility cap 12%: a name this wild shrinks a fixed-risk position to a token</t>
         </is>
       </c>
-      <c r="Z14" s="25" t="inlineStr"/>
+      <c r="Z14" s="25" t="n"/>
       <c r="AA14" s="25" t="inlineStr"/>
+      <c r="AB14" s="25" t="inlineStr"/>
     </row>
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="23" t="n">
@@ -34260,8 +34291,9 @@
           <t>trend strength (ADX) 17.7118 below 20 - no trend to ride</t>
         </is>
       </c>
-      <c r="Z15" s="25" t="inlineStr"/>
+      <c r="Z15" s="25" t="n"/>
       <c r="AA15" s="25" t="inlineStr"/>
+      <c r="AB15" s="25" t="inlineStr"/>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="23" t="n">
@@ -34359,8 +34391,9 @@
           <t>stop is 0.88x ATR (2.8687) - inside daily noise, it gets hit by nothing happening (floor 1.0x)</t>
         </is>
       </c>
-      <c r="Z16" s="25" t="inlineStr"/>
+      <c r="Z16" s="25" t="n"/>
       <c r="AA16" s="25" t="inlineStr"/>
+      <c r="AB16" s="25" t="inlineStr"/>
     </row>
     <row r="17" ht="60" customHeight="1">
       <c r="A17" s="23" t="n">
@@ -34452,8 +34485,9 @@
           <t>trend strength (ADX) 19.0248 below 20 - no trend to ride; stop is 5.37x ATR (multiples of a normal day's swing) - so wide the position shrinks to a token (ceili...</t>
         </is>
       </c>
-      <c r="Z17" s="25" t="inlineStr"/>
+      <c r="Z17" s="25" t="n"/>
       <c r="AA17" s="25" t="inlineStr"/>
+      <c r="AB17" s="25" t="inlineStr"/>
     </row>
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="23" t="n">
@@ -34545,8 +34579,9 @@
           <t>stop is 12.9% away - volatility cap 12%: a name this wild shrinks a fixed-risk position to a token</t>
         </is>
       </c>
-      <c r="Z18" s="25" t="inlineStr"/>
+      <c r="Z18" s="25" t="n"/>
       <c r="AA18" s="25" t="inlineStr"/>
+      <c r="AB18" s="25" t="inlineStr"/>
     </row>
     <row r="19" ht="45" customHeight="1">
       <c r="A19" s="23" t="n">
@@ -34644,8 +34679,9 @@
           <t>trend strength (ADX) 19.2408 below 20 - no trend to ride; stop is 13.5% away - volatility cap 12%: a name this wild shrinks ...</t>
         </is>
       </c>
-      <c r="Z19" s="25" t="inlineStr"/>
+      <c r="Z19" s="25" t="n"/>
       <c r="AA19" s="25" t="inlineStr"/>
+      <c r="AB19" s="25" t="inlineStr"/>
     </row>
     <row r="20" ht="45" customHeight="1">
       <c r="A20" s="23" t="n">
@@ -34737,8 +34773,9 @@
           <t>trend strength (ADX) 15.9956 below 20 - no trend to ride</t>
         </is>
       </c>
-      <c r="Z20" s="25" t="inlineStr"/>
+      <c r="Z20" s="25" t="n"/>
       <c r="AA20" s="25" t="inlineStr"/>
+      <c r="AB20" s="25" t="inlineStr"/>
     </row>
     <row r="21" ht="45" customHeight="1">
       <c r="A21" s="23" t="n">
@@ -34830,8 +34867,9 @@
           <t>-DI 22.8119 &gt;= +DI 17.973 - sellers in control; stop is 18.9% away - volatility cap 12%: a name this wild s...</t>
         </is>
       </c>
-      <c r="Z21" s="25" t="inlineStr"/>
+      <c r="Z21" s="25" t="n"/>
       <c r="AA21" s="25" t="inlineStr"/>
+      <c r="AB21" s="25" t="inlineStr"/>
     </row>
     <row r="22" ht="45" customHeight="1">
       <c r="A22" s="23" t="n">
@@ -34923,8 +34961,9 @@
           <t>regime DEEP-FAIL (-19.1307% vs the 200-day average) - watch only, no size</t>
         </is>
       </c>
-      <c r="Z22" s="25" t="inlineStr"/>
+      <c r="Z22" s="25" t="n"/>
       <c r="AA22" s="25" t="inlineStr"/>
+      <c r="AB22" s="25" t="inlineStr"/>
     </row>
     <row r="23" ht="45" customHeight="1">
       <c r="A23" s="23" t="n">
@@ -35016,8 +35055,9 @@
           <t>regime DEEP-FAIL (-21.3289% vs the 200-day average) - watch only, no size; -DI 21.5394 &gt;= +DI 15.2549 - sellers in control</t>
         </is>
       </c>
-      <c r="Z23" s="25" t="inlineStr"/>
+      <c r="Z23" s="25" t="n"/>
       <c r="AA23" s="25" t="inlineStr"/>
+      <c r="AB23" s="25" t="inlineStr"/>
     </row>
     <row r="24" ht="45" customHeight="1">
       <c r="A24" s="23" t="n">
@@ -35115,8 +35155,9 @@
           <t>-DI 19.8414 &gt;= +DI 18.5857 - sellers in control; stop is 15.2% away - volatility cap 12%: a name this wild ...</t>
         </is>
       </c>
-      <c r="Z24" s="25" t="inlineStr"/>
+      <c r="Z24" s="25" t="n"/>
       <c r="AA24" s="25" t="inlineStr"/>
+      <c r="AB24" s="25" t="inlineStr"/>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="23" t="n">
@@ -35198,8 +35239,9 @@
           <t>stop is 0.94x ATR (0.9547) - inside daily noise, it gets hit by nothing happening (floor 1.0x)</t>
         </is>
       </c>
-      <c r="Z25" s="25" t="inlineStr"/>
+      <c r="Z25" s="25" t="n"/>
       <c r="AA25" s="25" t="inlineStr"/>
+      <c r="AB25" s="25" t="inlineStr"/>
     </row>
     <row r="26" ht="45" customHeight="1">
       <c r="A26" s="23" t="n">
@@ -35291,8 +35333,9 @@
           <t>trend strength (ADX) 19.4768 below 20 - no trend to ride; stop is 0.85x ATR (13.4615) - inside daily noise, it gets hit by n...</t>
         </is>
       </c>
-      <c r="Z26" s="25" t="inlineStr"/>
+      <c r="Z26" s="25" t="n"/>
       <c r="AA26" s="25" t="inlineStr"/>
+      <c r="AB26" s="25" t="inlineStr"/>
     </row>
     <row r="27" ht="45" customHeight="1">
       <c r="A27" s="23" t="n">
@@ -35384,8 +35427,9 @@
           <t>stop is 12.3% away - volatility cap 12%: a name this wild shrinks a fixed-risk position to a token</t>
         </is>
       </c>
-      <c r="Z27" s="25" t="inlineStr"/>
+      <c r="Z27" s="25" t="n"/>
       <c r="AA27" s="25" t="inlineStr"/>
+      <c r="AB27" s="25" t="inlineStr"/>
     </row>
     <row r="28" ht="60" customHeight="1">
       <c r="A28" s="23" t="n">
@@ -35477,12 +35521,13 @@
           <t>regime DEEP-FAIL (-29.1609% vs the 200-day average) - watch only, no size</t>
         </is>
       </c>
-      <c r="Z28" s="25" t="inlineStr">
+      <c r="Z28" s="25" t="n"/>
+      <c r="AA28" s="25" t="inlineStr">
         <is>
           <t>Earnings 2026-08-04</t>
         </is>
       </c>
-      <c r="AA28" s="25" t="inlineStr">
+      <c r="AB28" s="25" t="inlineStr">
         <is>
           <t>Reports 2026-08-04 (est EPS +2.91). If long &amp; extended, TRIM into the print - do NOT hold full size through a binary. Fresh entry only POST-print if it beats AND holds the gap (PEAD drift = our one measured edge); else awareness-only.</t>
         </is>
@@ -35584,8 +35629,9 @@
           <t>trend strength (ADX) 17.5543 below 20 - no trend to ride; -DI 22.6262 &gt;= +DI 13.9685 - sellers in control; stop is 0.94x ATR (multiples of a normal day's swing)...</t>
         </is>
       </c>
-      <c r="Z29" s="25" t="inlineStr"/>
+      <c r="Z29" s="25" t="n"/>
       <c r="AA29" s="25" t="inlineStr"/>
+      <c r="AB29" s="25" t="inlineStr"/>
     </row>
     <row r="30" ht="45" customHeight="1">
       <c r="A30" s="23" t="n">
@@ -35683,8 +35729,9 @@
           <t>price 145.1075 at/below its trend line (ZLSMA) 148.9537 - structure has not turned</t>
         </is>
       </c>
-      <c r="Z30" s="25" t="inlineStr"/>
+      <c r="Z30" s="25" t="n"/>
       <c r="AA30" s="25" t="inlineStr"/>
+      <c r="AB30" s="25" t="inlineStr"/>
     </row>
     <row r="31" ht="45" customHeight="1">
       <c r="A31" s="23" t="n">
@@ -35776,8 +35823,9 @@
           <t>trend strength (ADX) 18.9553 below 20 - no trend to ride</t>
         </is>
       </c>
-      <c r="Z31" s="25" t="inlineStr"/>
+      <c r="Z31" s="25" t="n"/>
       <c r="AA31" s="25" t="inlineStr"/>
+      <c r="AB31" s="25" t="inlineStr"/>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="23" t="n">
@@ -35869,8 +35917,9 @@
           <t>trend strength (ADX) 19.9053 below 20 - no trend to ride</t>
         </is>
       </c>
-      <c r="Z32" s="25" t="inlineStr"/>
+      <c r="Z32" s="25" t="n"/>
       <c r="AA32" s="25" t="inlineStr"/>
+      <c r="AB32" s="25" t="inlineStr"/>
     </row>
     <row r="33" ht="45" customHeight="1">
       <c r="A33" s="23" t="n">
@@ -35962,8 +36011,9 @@
           <t>regime DEEP-FAIL (-16.4329% vs the 200-day average) - watch only, no size; stop is 13.9% away - volatility cap 12%: a n...</t>
         </is>
       </c>
-      <c r="Z33" s="25" t="inlineStr"/>
+      <c r="Z33" s="25" t="n"/>
       <c r="AA33" s="25" t="inlineStr"/>
+      <c r="AB33" s="25" t="inlineStr"/>
     </row>
     <row r="34" ht="60" customHeight="1">
       <c r="A34" s="23" t="n">
@@ -36055,12 +36105,13 @@
           <t>regime DEEP-FAIL (-10.0651% vs the 200-day average) - watch only, no size; trend strength (ADX) 18.4779 below 20 - no trend to ride</t>
         </is>
       </c>
-      <c r="Z34" s="25" t="inlineStr">
+      <c r="Z34" s="25" t="n"/>
+      <c r="AA34" s="25" t="inlineStr">
         <is>
           <t>Earnings 2026-08-06</t>
         </is>
       </c>
-      <c r="AA34" s="25" t="inlineStr">
+      <c r="AB34" s="25" t="inlineStr">
         <is>
           <t>Reports 2026-08-06 (est EPS +2.89). If long &amp; extended, TRIM into the print - do NOT hold full size through a binary. Fresh entry only POST-print if it beats AND holds the gap (PEAD drift = our one measured edge); else awareness-only.</t>
         </is>
@@ -36162,8 +36213,9 @@
           <t>trend strength (ADX) 19.4184 below 20 - no trend to ride</t>
         </is>
       </c>
-      <c r="Z35" s="25" t="inlineStr"/>
+      <c r="Z35" s="25" t="n"/>
       <c r="AA35" s="25" t="inlineStr"/>
+      <c r="AB35" s="25" t="inlineStr"/>
     </row>
     <row r="36" ht="45" customHeight="1">
       <c r="A36" s="23" t="n">
@@ -36245,8 +36297,9 @@
           <t>trend strength (ADX) 18.9276 below 20 - no trend to ride</t>
         </is>
       </c>
-      <c r="Z36" s="25" t="inlineStr"/>
+      <c r="Z36" s="25" t="n"/>
       <c r="AA36" s="25" t="inlineStr"/>
+      <c r="AB36" s="25" t="inlineStr"/>
     </row>
     <row r="37" ht="45" customHeight="1">
       <c r="A37" s="23" t="n">
@@ -36338,8 +36391,9 @@
           <t>regime DEEP-FAIL (-18.0618% vs the 200-day average) - watch only, no size; -DI 23.8609 &gt;= +DI 14.7481 - sellers in cont...</t>
         </is>
       </c>
-      <c r="Z37" s="25" t="inlineStr"/>
+      <c r="Z37" s="25" t="n"/>
       <c r="AA37" s="25" t="inlineStr"/>
+      <c r="AB37" s="25" t="inlineStr"/>
     </row>
     <row r="38" ht="45" customHeight="1">
       <c r="A38" s="23" t="n">
@@ -36431,8 +36485,9 @@
           <t>regime DEEP-FAIL (-25.9228% vs the 200-day average) - watch only, no size; trend strength (ADX) 16.5719 below 20 - no trend to ride</t>
         </is>
       </c>
-      <c r="Z38" s="25" t="inlineStr"/>
+      <c r="Z38" s="25" t="n"/>
       <c r="AA38" s="25" t="inlineStr"/>
+      <c r="AB38" s="25" t="inlineStr"/>
     </row>
     <row r="39" ht="45" customHeight="1">
       <c r="A39" s="23" t="n">
@@ -36514,8 +36569,9 @@
           <t>trend strength (ADX) 11.5189 below 20 - no trend to ride</t>
         </is>
       </c>
-      <c r="Z39" s="25" t="inlineStr"/>
+      <c r="Z39" s="25" t="n"/>
       <c r="AA39" s="25" t="inlineStr"/>
+      <c r="AB39" s="25" t="inlineStr"/>
     </row>
     <row r="40" ht="45" customHeight="1">
       <c r="A40" s="23" t="n">
@@ -36613,8 +36669,9 @@
           <t>price 17.075 at/below its trend line (ZLSMA) 18.102 - structure has not turned</t>
         </is>
       </c>
-      <c r="Z40" s="25" t="inlineStr"/>
+      <c r="Z40" s="25" t="n"/>
       <c r="AA40" s="25" t="inlineStr"/>
+      <c r="AB40" s="25" t="inlineStr"/>
     </row>
     <row r="41" ht="45" customHeight="1">
       <c r="A41" s="23" t="n">
@@ -36706,8 +36763,9 @@
           <t>regime DEEP-FAIL (-12.4149% vs the 200-day average) - watch only, no size; trend strength (ADX) 17.1454 below 20 - no trend to ride</t>
         </is>
       </c>
-      <c r="Z41" s="25" t="inlineStr"/>
+      <c r="Z41" s="25" t="n"/>
       <c r="AA41" s="25" t="inlineStr"/>
+      <c r="AB41" s="25" t="inlineStr"/>
     </row>
     <row r="42" ht="60" customHeight="1">
       <c r="A42" s="23" t="n">
@@ -36805,12 +36863,13 @@
           <t>trend strength (ADX) 15.3446 below 20 - no trend to ride; -DI 17.2802 &gt;= +DI 16.2219 - sellers in control</t>
         </is>
       </c>
-      <c r="Z42" s="25" t="inlineStr">
+      <c r="Z42" s="25" t="n"/>
+      <c r="AA42" s="25" t="inlineStr">
         <is>
           <t>Earnings 2026-08-03</t>
         </is>
       </c>
-      <c r="AA42" s="25" t="inlineStr">
+      <c r="AB42" s="25" t="inlineStr">
         <is>
           <t>Reports 2026-08-03 (est EPS +3.08). If long &amp; extended, TRIM into the print - do NOT hold full size through a binary. Fresh entry only POST-print if it beats AND holds the gap (PEAD drift = our one measured edge); else awareness-only.</t>
         </is>
@@ -36906,12 +36965,13 @@
           <t>price 32.2557 at/below its trend line (ZLSMA) 33.6072 - structure has not turned</t>
         </is>
       </c>
-      <c r="Z43" s="25" t="inlineStr">
+      <c r="Z43" s="25" t="n"/>
+      <c r="AA43" s="25" t="inlineStr">
         <is>
           <t>Earnings 2026-08-04</t>
         </is>
       </c>
-      <c r="AA43" s="25" t="inlineStr">
+      <c r="AB43" s="25" t="inlineStr">
         <is>
           <t>Reports 2026-08-04 (est EPS +0.32). If long &amp; extended, TRIM into the print - do NOT hold full size through a binary. Fresh entry only POST-print if it beats AND holds the gap (PEAD drift = our one measured edge); else awareness-only.</t>
         </is>
@@ -37007,8 +37067,9 @@
           <t>price 248.34 at/below its trend line (ZLSMA) 267.7119 - structure has not turned</t>
         </is>
       </c>
-      <c r="Z44" s="25" t="inlineStr"/>
+      <c r="Z44" s="25" t="n"/>
       <c r="AA44" s="25" t="inlineStr"/>
+      <c r="AB44" s="25" t="inlineStr"/>
     </row>
     <row r="45" ht="60" customHeight="1">
       <c r="A45" s="23" t="n">
@@ -37100,12 +37161,13 @@
           <t>regime DEEP-FAIL (-10.6727% vs the 200-day average) - watch only, no size; trend strength (ADX) 16.1533 below 20 - no trend to ride; sto...</t>
         </is>
       </c>
-      <c r="Z45" s="25" t="inlineStr">
+      <c r="Z45" s="25" t="n"/>
+      <c r="AA45" s="25" t="inlineStr">
         <is>
           <t>Earnings 2026-08-04</t>
         </is>
       </c>
-      <c r="AA45" s="25" t="inlineStr">
+      <c r="AB45" s="25" t="inlineStr">
         <is>
           <t>Reports 2026-08-04 (est EPS +3.32). If long &amp; extended, TRIM into the print - do NOT hold full size through a binary. Fresh entry only POST-print if it beats AND holds the gap (PEAD drift = our one measured edge); else awareness-only.</t>
         </is>
@@ -37201,8 +37263,9 @@
           <t>regime DEEP-FAIL (-19.7291% vs the 200-day average) - watch only, no size; trend strength (ADX) 17.6438 below 20 - no trend to ride; sto...</t>
         </is>
       </c>
-      <c r="Z46" s="25" t="inlineStr"/>
+      <c r="Z46" s="25" t="n"/>
       <c r="AA46" s="25" t="inlineStr"/>
+      <c r="AB46" s="25" t="inlineStr"/>
     </row>
     <row r="47" ht="60" customHeight="1">
       <c r="A47" s="23" t="n">
@@ -37300,12 +37363,13 @@
           <t>price 129.575 at/below its trend line (ZLSMA) 129.7069 - structure has not turned</t>
         </is>
       </c>
-      <c r="Z47" s="25" t="inlineStr">
+      <c r="Z47" s="25" t="n"/>
+      <c r="AA47" s="25" t="inlineStr">
         <is>
           <t>Earnings 2026-08-04</t>
         </is>
       </c>
-      <c r="AA47" s="25" t="inlineStr">
+      <c r="AB47" s="25" t="inlineStr">
         <is>
           <t>Reports 2026-08-04 (est EPS -0.27). If long &amp; extended, TRIM into the print - do NOT hold full size through a binary. Fresh entry only POST-print if it beats AND holds the gap (PEAD drift = our one measured edge); else awareness-only.</t>
         </is>
@@ -37401,8 +37465,9 @@
           <t>price 100.5175 at/below its trend line (ZLSMA) 107.1078 - structure has not turned; stop is 0.74x ATR (multiples of a normal day's swing) (3.2018) - inside dail...</t>
         </is>
       </c>
-      <c r="Z48" s="25" t="inlineStr"/>
+      <c r="Z48" s="25" t="n"/>
       <c r="AA48" s="25" t="inlineStr"/>
+      <c r="AB48" s="25" t="inlineStr"/>
     </row>
     <row r="49" ht="45" customHeight="1">
       <c r="A49" s="23" t="n">
@@ -37494,8 +37559,9 @@
           <t>price 151.1525 at/below its trend line (ZLSMA) 154.0157 - structure has not turned</t>
         </is>
       </c>
-      <c r="Z49" s="25" t="inlineStr"/>
+      <c r="Z49" s="25" t="n"/>
       <c r="AA49" s="25" t="inlineStr"/>
+      <c r="AB49" s="25" t="inlineStr"/>
     </row>
     <row r="50" ht="45" customHeight="1">
       <c r="A50" s="23" t="n">
@@ -37577,8 +37643,9 @@
           <t>regime DEEP-FAIL (-11.3595% vs the 200-day average) - watch only, no size; price 28.31 at/below its trend line (ZLSMA) 28.5005 - structu...</t>
         </is>
       </c>
-      <c r="Z50" s="25" t="inlineStr"/>
+      <c r="Z50" s="25" t="n"/>
       <c r="AA50" s="25" t="inlineStr"/>
+      <c r="AB50" s="25" t="inlineStr"/>
     </row>
     <row r="51" ht="45" customHeight="1">
       <c r="A51" s="23" t="n">
@@ -37670,8 +37737,9 @@
           <t>price 387.9925 at/below its trend line (ZLSMA) 394.2479 - structure has not turned</t>
         </is>
       </c>
-      <c r="Z51" s="25" t="inlineStr"/>
+      <c r="Z51" s="25" t="n"/>
       <c r="AA51" s="25" t="inlineStr"/>
+      <c r="AB51" s="25" t="inlineStr"/>
     </row>
     <row r="52" ht="60" customHeight="1">
       <c r="A52" s="23" t="n">
@@ -37769,8 +37837,9 @@
           <t>price 133.165 at/below its trend line (ZLSMA) 133.5495 - structure has not turned; stop is 0.78x ATR (multiples of a normal day's swing) (4.5202) - inside daily...</t>
         </is>
       </c>
-      <c r="Z52" s="25" t="inlineStr"/>
+      <c r="Z52" s="25" t="n"/>
       <c r="AA52" s="25" t="inlineStr"/>
+      <c r="AB52" s="25" t="inlineStr"/>
     </row>
     <row r="53" ht="45" customHeight="1">
       <c r="A53" s="23" t="n">
@@ -37852,8 +37921,9 @@
           <t>regime DEEP-FAIL (-14.2162% vs the 200-day average) - watch only, no size; price 121.0413 at/below its trend line (ZLSMA) 121.9243 - str...</t>
         </is>
       </c>
-      <c r="Z53" s="25" t="inlineStr"/>
+      <c r="Z53" s="25" t="n"/>
       <c r="AA53" s="25" t="inlineStr"/>
+      <c r="AB53" s="25" t="inlineStr"/>
     </row>
     <row r="54" ht="60" customHeight="1">
       <c r="A54" s="23" t="n">
@@ -37951,8 +38021,9 @@
           <t>price 596.5877 at/below its trend line (ZLSMA) 627.1908 - structure has not turned; stop is 0.29x ATR (multiples of a normal day's swing) (21.3648) - inside dai...</t>
         </is>
       </c>
-      <c r="Z54" s="25" t="inlineStr"/>
+      <c r="Z54" s="25" t="n"/>
       <c r="AA54" s="25" t="inlineStr"/>
+      <c r="AB54" s="25" t="inlineStr"/>
     </row>
     <row r="55" ht="60" customHeight="1">
       <c r="A55" s="23" t="n">
@@ -38044,12 +38115,13 @@
           <t>price 133.0125 at/below its trend line (ZLSMA) 133.9452 - structure has not turned</t>
         </is>
       </c>
-      <c r="Z55" s="25" t="inlineStr">
+      <c r="Z55" s="25" t="n"/>
+      <c r="AA55" s="25" t="inlineStr">
         <is>
           <t>Earnings 2026-08-05</t>
         </is>
       </c>
-      <c r="AA55" s="25" t="inlineStr">
+      <c r="AB55" s="25" t="inlineStr">
         <is>
           <t>Reports 2026-08-05 (est EPS +0.60). If long &amp; extended, TRIM into the print - do NOT hold full size through a binary. Fresh entry only POST-print if it beats AND holds the gap (PEAD drift = our one measured edge); else awareness-only.</t>
         </is>
@@ -38151,8 +38223,9 @@
           <t>trend strength (ADX) 15.0931 below 20 - no trend to ride; price 296.8964 at/below its trend line (ZLSMA) 311.9719 - structure has not turned</t>
         </is>
       </c>
-      <c r="Z56" s="25" t="inlineStr"/>
+      <c r="Z56" s="25" t="n"/>
       <c r="AA56" s="25" t="inlineStr"/>
+      <c r="AB56" s="25" t="inlineStr"/>
     </row>
     <row r="57" ht="45" customHeight="1">
       <c r="A57" s="23" t="n">
@@ -38250,8 +38323,9 @@
           <t>trend strength (ADX) 19.2905 below 20 - no trend to ride; price 39.64 at/below its trend line (ZLSMA) 39.8437 - structure has not turned; sto...</t>
         </is>
       </c>
-      <c r="Z57" s="25" t="inlineStr"/>
+      <c r="Z57" s="25" t="n"/>
       <c r="AA57" s="25" t="inlineStr"/>
+      <c r="AB57" s="25" t="inlineStr"/>
     </row>
     <row r="58" ht="45" customHeight="1">
       <c r="A58" s="23" t="n">
@@ -38343,8 +38417,9 @@
           <t>price 85.1313 at/below its trend line (ZLSMA) 85.5862 - structure has not turned</t>
         </is>
       </c>
-      <c r="Z58" s="25" t="inlineStr"/>
+      <c r="Z58" s="25" t="n"/>
       <c r="AA58" s="25" t="inlineStr"/>
+      <c r="AB58" s="25" t="inlineStr"/>
     </row>
     <row r="59" ht="45" customHeight="1">
       <c r="A59" s="23" t="n">
@@ -38442,8 +38517,9 @@
           <t>-DI 19.2266 &gt;= +DI 18.3181 - sellers in control; price 10.7 at/below its trend line (ZLSMA) 11.3595 - structure has not turn...</t>
         </is>
       </c>
-      <c r="Z59" s="25" t="inlineStr"/>
+      <c r="Z59" s="25" t="n"/>
       <c r="AA59" s="25" t="inlineStr"/>
+      <c r="AB59" s="25" t="inlineStr"/>
     </row>
     <row r="60" ht="60" customHeight="1">
       <c r="A60" s="23" t="n">
@@ -38535,12 +38611,13 @@
           <t>price 196.435 at/below its trend line (ZLSMA) 201.9239 - structure has not turned</t>
         </is>
       </c>
-      <c r="Z60" s="25" t="inlineStr">
+      <c r="Z60" s="25" t="n"/>
+      <c r="AA60" s="25" t="inlineStr">
         <is>
           <t>Earnings 2026-08-05</t>
         </is>
       </c>
-      <c r="AA60" s="25" t="inlineStr">
+      <c r="AB60" s="25" t="inlineStr">
         <is>
           <t>Reports 2026-08-05 (est EPS +0.47). If long &amp; extended, TRIM into the print - do NOT hold full size through a binary. Fresh entry only POST-print if it beats AND holds the gap (PEAD drift = our one measured edge); else awareness-only.</t>
         </is>
@@ -38642,8 +38719,9 @@
           <t>-DI 21.6818 &gt;= +DI 16.4664 - sellers in control; price 179.3075 at/below its trend line (ZLSMA) 183.5418 - structure has not...</t>
         </is>
       </c>
-      <c r="Z61" s="25" t="inlineStr"/>
+      <c r="Z61" s="25" t="n"/>
       <c r="AA61" s="25" t="inlineStr"/>
+      <c r="AB61" s="25" t="inlineStr"/>
     </row>
     <row r="62" ht="60" customHeight="1">
       <c r="A62" s="23" t="n">
@@ -38735,12 +38813,13 @@
           <t>trend strength (ADX) 16.1122 below 20 - no trend to ride; price 188.3075 at/below its trend line (ZLSMA) 189.3949 - structure has not turned</t>
         </is>
       </c>
-      <c r="Z62" s="25" t="inlineStr">
+      <c r="Z62" s="25" t="n"/>
+      <c r="AA62" s="25" t="inlineStr">
         <is>
           <t>Earnings 2026-08-05</t>
         </is>
       </c>
-      <c r="AA62" s="25" t="inlineStr">
+      <c r="AB62" s="25" t="inlineStr">
         <is>
           <t>Reports 2026-08-05 (est EPS n/a). If long &amp; extended, TRIM into the print - do NOT hold full size through a binary. Fresh entry only POST-print if it beats AND holds the gap (PEAD drift = our one measured edge); else awareness-only.</t>
         </is>
@@ -38836,8 +38915,9 @@
           <t>price 341.1725 at/below its trend line (ZLSMA) 345.7113 - structure has not turned; stop is 0.74x ATR (multiples of a normal day's swing) (13.1473) - inside dai...</t>
         </is>
       </c>
-      <c r="Z63" s="25" t="inlineStr"/>
+      <c r="Z63" s="25" t="n"/>
       <c r="AA63" s="25" t="inlineStr"/>
+      <c r="AB63" s="25" t="inlineStr"/>
     </row>
     <row r="64" ht="60" customHeight="1">
       <c r="A64" s="23" t="n">
@@ -38929,8 +39009,9 @@
           <t>price 211.5075 at/below its trend line (ZLSMA) 218.7627 - structure has not turned; stop is 0.78x ATR (multiples of a normal day's swing) (9.071) - inside daily...</t>
         </is>
       </c>
-      <c r="Z64" s="25" t="inlineStr"/>
+      <c r="Z64" s="25" t="n"/>
       <c r="AA64" s="25" t="inlineStr"/>
+      <c r="AB64" s="25" t="inlineStr"/>
     </row>
     <row r="65" ht="45" customHeight="1">
       <c r="A65" s="23" t="n">
@@ -39028,8 +39109,9 @@
           <t>trend strength (ADX) 16.9636 below 20 - no trend to ride; -DI 20.7364 &gt;= +DI 18.12 - sellers in control; price 350.3325 at/b...</t>
         </is>
       </c>
-      <c r="Z65" s="25" t="inlineStr"/>
+      <c r="Z65" s="25" t="n"/>
       <c r="AA65" s="25" t="inlineStr"/>
+      <c r="AB65" s="25" t="inlineStr"/>
     </row>
     <row r="66" ht="60" customHeight="1">
       <c r="A66" s="23" t="n">
@@ -39121,12 +39203,13 @@
           <t>price 523.136 at/below its trend line (ZLSMA) 535.5478 - structure has not turned; stop is 0.97x ATR (multiples of a normal day's swing) (33.2767) - inside dail...</t>
         </is>
       </c>
-      <c r="Z66" s="25" t="inlineStr">
+      <c r="Z66" s="25" t="n"/>
+      <c r="AA66" s="25" t="inlineStr">
         <is>
           <t>Earnings 2026-08-05</t>
         </is>
       </c>
-      <c r="AA66" s="25" t="inlineStr">
+      <c r="AB66" s="25" t="inlineStr">
         <is>
           <t>Reports 2026-08-05 (est EPS +1.84). If long &amp; extended, TRIM into the print - do NOT hold full size through a binary. Fresh entry only POST-print if it beats AND holds the gap (PEAD drift = our one measured edge); else awareness-only.</t>
         </is>
@@ -39222,12 +39305,13 @@
           <t>regime DEEP-FAIL (-23.1574% vs the 200-day average) - watch only, no size; price 63.0125 at/below its trend line (ZLSMA) 69.9927 - struc...</t>
         </is>
       </c>
-      <c r="Z67" s="25" t="inlineStr">
+      <c r="Z67" s="25" t="n"/>
+      <c r="AA67" s="25" t="inlineStr">
         <is>
           <t>Earnings 2026-08-05</t>
         </is>
       </c>
-      <c r="AA67" s="25" t="inlineStr">
+      <c r="AB67" s="25" t="inlineStr">
         <is>
           <t>Reports 2026-08-05 (est EPS +0.31). If long &amp; extended, TRIM into the print - do NOT hold full size through a binary. Fresh entry only POST-print if it beats AND holds the gap (PEAD drift = our one measured edge); else awareness-only.</t>
         </is>
@@ -39329,8 +39413,9 @@
           <t>trend strength (ADX) 16.123 below 20 - no trend to ride; -DI 16.4196 &gt;= +DI 15.6242 - sellers in control; price 971.9825 at/...</t>
         </is>
       </c>
-      <c r="Z68" s="25" t="inlineStr"/>
+      <c r="Z68" s="25" t="n"/>
       <c r="AA68" s="25" t="inlineStr"/>
+      <c r="AB68" s="25" t="inlineStr"/>
     </row>
     <row r="69" ht="45" customHeight="1">
       <c r="A69" s="23" t="n">
@@ -39422,8 +39507,9 @@
           <t>price 139.405 at/below its trend line (ZLSMA) 140.6837 - structure has not turned</t>
         </is>
       </c>
-      <c r="Z69" s="25" t="inlineStr"/>
+      <c r="Z69" s="25" t="n"/>
       <c r="AA69" s="25" t="inlineStr"/>
+      <c r="AB69" s="25" t="inlineStr"/>
     </row>
     <row r="70" ht="60" customHeight="1">
       <c r="A70" s="23" t="n">
@@ -39521,8 +39607,9 @@
           <t>price 186.8038 at/below its trend line (ZLSMA) 189.1902 - structure has not turned; stop is 0.44x ATR (multiples of a normal day's swing) (7.4025) - inside dail...</t>
         </is>
       </c>
-      <c r="Z70" s="25" t="inlineStr"/>
+      <c r="Z70" s="25" t="n"/>
       <c r="AA70" s="25" t="inlineStr"/>
+      <c r="AB70" s="25" t="inlineStr"/>
     </row>
     <row r="71" ht="45" customHeight="1">
       <c r="A71" s="23" t="n">
@@ -39620,8 +39707,9 @@
           <t>-DI 21.4858 &gt;= +DI 18.3012 - sellers in control; price 111.17 at/below its trend line (ZLSMA) 112.5104 - structure has not t...</t>
         </is>
       </c>
-      <c r="Z71" s="25" t="inlineStr"/>
+      <c r="Z71" s="25" t="n"/>
       <c r="AA71" s="25" t="inlineStr"/>
+      <c r="AB71" s="25" t="inlineStr"/>
     </row>
     <row r="72" ht="45" customHeight="1">
       <c r="A72" s="23" t="n">
@@ -39713,8 +39801,9 @@
           <t>regime DEEP-FAIL (-16.4518% vs the 200-day average) - watch only, no size; trend strength (ADX) 18.6733 below 20 - no trend to ride; pri...</t>
         </is>
       </c>
-      <c r="Z72" s="25" t="inlineStr"/>
+      <c r="Z72" s="25" t="n"/>
       <c r="AA72" s="25" t="inlineStr"/>
+      <c r="AB72" s="25" t="inlineStr"/>
     </row>
     <row r="73" ht="45" customHeight="1">
       <c r="A73" s="23" t="n">
@@ -39806,8 +39895,9 @@
           <t>trend strength (ADX) 10.1704 below 20 - no trend to ride; price 21.8037 at/below its trend line (ZLSMA) 22.658 - structure has not turned</t>
         </is>
       </c>
-      <c r="Z73" s="25" t="inlineStr"/>
+      <c r="Z73" s="25" t="n"/>
       <c r="AA73" s="25" t="inlineStr"/>
+      <c r="AB73" s="25" t="inlineStr"/>
     </row>
     <row r="74" ht="45" customHeight="1">
       <c r="A74" s="23" t="n">
@@ -39889,8 +39979,9 @@
           <t>regime DEEP-FAIL (-11.8072% vs the 200-day average) - watch only, no size; price 4.875 at/below its trend line (ZLSMA) 4.9064 - structur...</t>
         </is>
       </c>
-      <c r="Z74" s="25" t="inlineStr"/>
+      <c r="Z74" s="25" t="n"/>
       <c r="AA74" s="25" t="inlineStr"/>
+      <c r="AB74" s="25" t="inlineStr"/>
     </row>
     <row r="75" ht="60" customHeight="1">
       <c r="A75" s="23" t="n">
@@ -39982,12 +40073,13 @@
           <t>trend strength (ADX) 11.9623 below 20 - no trend to ride; price 95.4125 at/below its trend line (ZLSMA) 95.4299 - structure has not turned; s...</t>
         </is>
       </c>
-      <c r="Z75" s="25" t="inlineStr">
+      <c r="Z75" s="25" t="n"/>
+      <c r="AA75" s="25" t="inlineStr">
         <is>
           <t>Earnings 2026-08-03</t>
         </is>
       </c>
-      <c r="AA75" s="25" t="inlineStr">
+      <c r="AB75" s="25" t="inlineStr">
         <is>
           <t>Reports 2026-08-03 (est EPS +1.64). If long &amp; extended, TRIM into the print - do NOT hold full size through a binary. Fresh entry only POST-print if it beats AND holds the gap (PEAD drift = our one measured edge); else awareness-only.</t>
         </is>
@@ -40083,8 +40175,9 @@
           <t>trend strength (ADX) 14.7655 below 20 - no trend to ride; -DI 18.0212 &gt;= +DI 17.4126 - sellers in control; price 331.7976 at...</t>
         </is>
       </c>
-      <c r="Z76" s="25" t="inlineStr"/>
+      <c r="Z76" s="25" t="n"/>
       <c r="AA76" s="25" t="inlineStr"/>
+      <c r="AB76" s="25" t="inlineStr"/>
     </row>
     <row r="77" ht="45" customHeight="1">
       <c r="A77" s="23" t="n">
@@ -40176,8 +40269,9 @@
           <t>trend strength (ADX) 13.8388 below 20 - no trend to ride; -DI 21.9574 &gt;= +DI 16.4501 - sellers in control; price 18.7225 at/...</t>
         </is>
       </c>
-      <c r="Z77" s="25" t="inlineStr"/>
+      <c r="Z77" s="25" t="n"/>
       <c r="AA77" s="25" t="inlineStr"/>
+      <c r="AB77" s="25" t="inlineStr"/>
     </row>
     <row r="78" ht="45" customHeight="1">
       <c r="A78" s="23" t="n">
@@ -40269,8 +40363,9 @@
           <t>regime DEEP-FAIL (-30.9453% vs the 200-day average) - watch only, no size; trend strength (ADX) 17.7745 below 20 - no trend to ride; -DI...</t>
         </is>
       </c>
-      <c r="Z78" s="25" t="inlineStr"/>
+      <c r="Z78" s="25" t="n"/>
       <c r="AA78" s="25" t="inlineStr"/>
+      <c r="AB78" s="25" t="inlineStr"/>
     </row>
     <row r="79" ht="45" customHeight="1">
       <c r="A79" s="23" t="n">
@@ -40362,11 +40457,12 @@
           <t>regime DEEP-FAIL (-13.1518% vs the 200-day average) - watch only, no size; trend strength (ADX) 16.3357 below 20 - no trend to ride; -DI...</t>
         </is>
       </c>
-      <c r="Z79" s="25" t="inlineStr"/>
+      <c r="Z79" s="25" t="n"/>
       <c r="AA79" s="25" t="inlineStr"/>
+      <c r="AB79" s="25" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AA1"/>
+  <autoFilter ref="A1:AB1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -40378,7 +40474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N41"/>
+  <dimension ref="A1:O41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -40393,8 +40489,9 @@
     <col width="11" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="44" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
-    <col width="62" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="62" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -40460,10 +40557,15 @@
       </c>
       <c r="M1" s="12" t="inlineStr">
         <is>
+          <t>Rested Leader</t>
+        </is>
+      </c>
+      <c r="N1" s="12" t="inlineStr">
+        <is>
           <t>Catalyst</t>
         </is>
       </c>
-      <c r="N1" s="12" t="inlineStr">
+      <c r="O1" s="12" t="inlineStr">
         <is>
           <t>Catalyst View</t>
         </is>
@@ -40514,12 +40616,13 @@
           <t>STARTER (regime REPAIR - half size). regime REPAIR (-3.5624% vs the 200-day average) - starter size only</t>
         </is>
       </c>
-      <c r="M2" s="19" t="inlineStr">
+      <c r="M2" s="19" t="n"/>
+      <c r="N2" s="19" t="inlineStr">
         <is>
           <t>Earnings 2026-08-04</t>
         </is>
       </c>
-      <c r="N2" s="19" t="inlineStr">
+      <c r="O2" s="19" t="inlineStr">
         <is>
           <t>Reports 2026-08-04 (est EPS +0.68). If long &amp; extended, TRIM into the print - do NOT hold full size through a binary. Fresh entry only POST-print if it beats AND holds the gap (PEAD drift = our one measured edge); else awareness-only.</t>
         </is>
@@ -40570,8 +40673,9 @@
           <t>STARTER (regime REPAIR - half size). regime REPAIR (-3.4519% vs the 200-day average) - starter size only</t>
         </is>
       </c>
-      <c r="M3" s="19" t="inlineStr"/>
+      <c r="M3" s="19" t="n"/>
       <c r="N3" s="19" t="inlineStr"/>
+      <c r="O3" s="19" t="inlineStr"/>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="17" t="n">
@@ -40618,8 +40722,9 @@
           <t>STARTER (regime REPAIR - half size). regime REPAIR (-1.0484% vs the 200-day average) - starter size only</t>
         </is>
       </c>
-      <c r="M4" s="19" t="inlineStr"/>
+      <c r="M4" s="19" t="n"/>
       <c r="N4" s="19" t="inlineStr"/>
+      <c r="O4" s="19" t="inlineStr"/>
     </row>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="17" t="n">
@@ -40666,8 +40771,9 @@
           <t>Passes every gate.</t>
         </is>
       </c>
-      <c r="M5" s="19" t="inlineStr"/>
+      <c r="M5" s="19" t="n"/>
       <c r="N5" s="19" t="inlineStr"/>
+      <c r="O5" s="19" t="inlineStr"/>
     </row>
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="17" t="n">
@@ -40714,12 +40820,13 @@
           <t>STARTER (regime REPAIR - half size). regime REPAIR (3.8185% vs the 200-day average) - starter size only</t>
         </is>
       </c>
-      <c r="M6" s="19" t="inlineStr">
+      <c r="M6" s="19" t="n"/>
+      <c r="N6" s="19" t="inlineStr">
         <is>
           <t>Earnings 2026-08-05</t>
         </is>
       </c>
-      <c r="N6" s="19" t="inlineStr">
+      <c r="O6" s="19" t="inlineStr">
         <is>
           <t>Reports 2026-08-05 (est EPS +3.85). If long &amp; extended, TRIM into the print - do NOT hold full size through a binary. Fresh entry only POST-print if it beats AND holds the gap (PEAD drift = our one measured edge); else awareness-only.</t>
         </is>
@@ -40770,8 +40877,9 @@
           <t>Passes every gate.</t>
         </is>
       </c>
-      <c r="M7" s="19" t="inlineStr"/>
+      <c r="M7" s="19" t="n"/>
       <c r="N7" s="19" t="inlineStr"/>
+      <c r="O7" s="19" t="inlineStr"/>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="17" t="n">
@@ -40818,8 +40926,9 @@
           <t>Passes every gate.</t>
         </is>
       </c>
-      <c r="M8" s="19" t="inlineStr"/>
+      <c r="M8" s="19" t="n"/>
       <c r="N8" s="19" t="inlineStr"/>
+      <c r="O8" s="19" t="inlineStr"/>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="17" t="n">
@@ -40866,8 +40975,9 @@
           <t>STARTER (regime REPAIR - half size). regime REPAIR (8.4497% vs the 200-day average) - starter size only</t>
         </is>
       </c>
-      <c r="M9" s="19" t="inlineStr"/>
+      <c r="M9" s="19" t="n"/>
       <c r="N9" s="19" t="inlineStr"/>
+      <c r="O9" s="19" t="inlineStr"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="17" t="n">
@@ -40914,8 +41024,9 @@
           <t>Passes every gate.</t>
         </is>
       </c>
-      <c r="M10" s="19" t="inlineStr"/>
+      <c r="M10" s="19" t="n"/>
       <c r="N10" s="19" t="inlineStr"/>
+      <c r="O10" s="19" t="inlineStr"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="17" t="n">
@@ -40962,8 +41073,9 @@
           <t>Passes every gate.</t>
         </is>
       </c>
-      <c r="M11" s="19" t="inlineStr"/>
+      <c r="M11" s="19" t="n"/>
       <c r="N11" s="19" t="inlineStr"/>
+      <c r="O11" s="19" t="inlineStr"/>
     </row>
     <row r="12" ht="45" customHeight="1">
       <c r="A12" s="17" t="n">
@@ -41010,8 +41122,9 @@
           <t>Passes every gate.</t>
         </is>
       </c>
-      <c r="M12" s="19" t="inlineStr"/>
+      <c r="M12" s="19" t="n"/>
       <c r="N12" s="19" t="inlineStr"/>
+      <c r="O12" s="19" t="inlineStr"/>
     </row>
     <row r="13" ht="60" customHeight="1">
       <c r="A13" s="17" t="n">
@@ -41058,12 +41171,13 @@
           <t>Passes every gate.</t>
         </is>
       </c>
-      <c r="M13" s="19" t="inlineStr">
+      <c r="M13" s="19" t="n"/>
+      <c r="N13" s="19" t="inlineStr">
         <is>
           <t>Earnings 2026-08-04</t>
         </is>
       </c>
-      <c r="N13" s="19" t="inlineStr">
+      <c r="O13" s="19" t="inlineStr">
         <is>
           <t>Reports 2026-08-04 (est EPS +5.62). If long &amp; extended, TRIM into the print - do NOT hold full size through a binary. Fresh entry only POST-print if it beats AND holds the gap (PEAD drift = our one measured edge); else awareness-only.</t>
         </is>
@@ -41114,8 +41228,9 @@
           <t>STARTER (regime REPAIR - half size). regime REPAIR (11.8104% vs the 200-day average) - starter size only</t>
         </is>
       </c>
-      <c r="M14" s="19" t="inlineStr"/>
+      <c r="M14" s="19" t="n"/>
       <c r="N14" s="19" t="inlineStr"/>
+      <c r="O14" s="19" t="inlineStr"/>
     </row>
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="17" t="n">
@@ -41162,8 +41277,13 @@
           <t>Passes every gate.</t>
         </is>
       </c>
-      <c r="M15" s="19" t="inlineStr"/>
+      <c r="M15" s="19" t="inlineStr">
+        <is>
+          <t>RESTED LEADER - on trial</t>
+        </is>
+      </c>
       <c r="N15" s="19" t="inlineStr"/>
+      <c r="O15" s="19" t="inlineStr"/>
     </row>
     <row r="16" ht="45" customHeight="1">
       <c r="A16" s="17" t="n">
@@ -41210,8 +41330,9 @@
           <t>Passes every gate.</t>
         </is>
       </c>
-      <c r="M16" s="19" t="inlineStr"/>
+      <c r="M16" s="19" t="n"/>
       <c r="N16" s="19" t="inlineStr"/>
+      <c r="O16" s="19" t="inlineStr"/>
     </row>
     <row r="17" ht="60" customHeight="1">
       <c r="A17" s="17" t="n">
@@ -41258,12 +41379,13 @@
           <t>Passes every gate.</t>
         </is>
       </c>
-      <c r="M17" s="19" t="inlineStr">
+      <c r="M17" s="19" t="n"/>
+      <c r="N17" s="19" t="inlineStr">
         <is>
           <t>Earnings 2026-08-04</t>
         </is>
       </c>
-      <c r="N17" s="19" t="inlineStr">
+      <c r="O17" s="19" t="inlineStr">
         <is>
           <t>Reports 2026-08-04 (est EPS +0.20). If long &amp; extended, TRIM into the print - do NOT hold full size through a binary. Fresh entry only POST-print if it beats AND holds the gap (PEAD drift = our one measured edge); else awareness-only.</t>
         </is>
@@ -41314,8 +41436,9 @@
           <t>Passes every gate.</t>
         </is>
       </c>
-      <c r="M18" s="19" t="inlineStr"/>
+      <c r="M18" s="19" t="n"/>
       <c r="N18" s="19" t="inlineStr"/>
+      <c r="O18" s="19" t="inlineStr"/>
     </row>
     <row r="19" ht="45" customHeight="1">
       <c r="A19" s="17" t="n">
@@ -41362,8 +41485,13 @@
           <t>Passes every gate.</t>
         </is>
       </c>
-      <c r="M19" s="19" t="inlineStr"/>
+      <c r="M19" s="19" t="inlineStr">
+        <is>
+          <t>RESTED LEADER - on trial</t>
+        </is>
+      </c>
       <c r="N19" s="19" t="inlineStr"/>
+      <c r="O19" s="19" t="inlineStr"/>
     </row>
     <row r="20" ht="45" customHeight="1">
       <c r="A20" s="17" t="n">
@@ -41410,8 +41538,9 @@
           <t>Passes every gate.</t>
         </is>
       </c>
-      <c r="M20" s="19" t="inlineStr"/>
+      <c r="M20" s="19" t="n"/>
       <c r="N20" s="19" t="inlineStr"/>
+      <c r="O20" s="19" t="inlineStr"/>
     </row>
     <row r="21" ht="60" customHeight="1">
       <c r="A21" s="17" t="n">
@@ -41458,12 +41587,13 @@
           <t>Passes every gate.</t>
         </is>
       </c>
-      <c r="M21" s="19" t="inlineStr">
+      <c r="M21" s="19" t="n"/>
+      <c r="N21" s="19" t="inlineStr">
         <is>
           <t>Earnings 2026-08-03</t>
         </is>
       </c>
-      <c r="N21" s="19" t="inlineStr">
+      <c r="O21" s="19" t="inlineStr">
         <is>
           <t>Reports 2026-08-03 (est EPS +6.08). If long &amp; extended, TRIM into the print - do NOT hold full size through a binary. Fresh entry only POST-print if it beats AND holds the gap (PEAD drift = our one measured edge); else awareness-only.</t>
         </is>
@@ -41514,12 +41644,13 @@
           <t>Passes every gate.</t>
         </is>
       </c>
-      <c r="M22" s="19" t="inlineStr">
+      <c r="M22" s="19" t="n"/>
+      <c r="N22" s="19" t="inlineStr">
         <is>
           <t>Earnings 2026-08-04</t>
         </is>
       </c>
-      <c r="N22" s="19" t="inlineStr">
+      <c r="O22" s="19" t="inlineStr">
         <is>
           <t>Reports 2026-08-04 (est EPS +5.00). If long &amp; extended, TRIM into the print - do NOT hold full size through a binary. Fresh entry only POST-print if it beats AND holds the gap (PEAD drift = our one measured edge); else awareness-only.</t>
         </is>
@@ -41570,8 +41701,9 @@
           <t>Passes every gate.</t>
         </is>
       </c>
-      <c r="M23" s="19" t="inlineStr"/>
+      <c r="M23" s="19" t="n"/>
       <c r="N23" s="19" t="inlineStr"/>
+      <c r="O23" s="19" t="inlineStr"/>
     </row>
     <row r="24" ht="45" customHeight="1">
       <c r="A24" s="17" t="n">
@@ -41618,8 +41750,9 @@
           <t>STARTER (regime REPAIR - half size). regime REPAIR (23.0346% vs the 200-day average) - starter size only</t>
         </is>
       </c>
-      <c r="M24" s="19" t="inlineStr"/>
+      <c r="M24" s="19" t="n"/>
       <c r="N24" s="19" t="inlineStr"/>
+      <c r="O24" s="19" t="inlineStr"/>
     </row>
     <row r="25" ht="45" customHeight="1">
       <c r="A25" s="17" t="n">
@@ -41666,8 +41799,9 @@
           <t>Passes every gate.</t>
         </is>
       </c>
-      <c r="M25" s="19" t="inlineStr"/>
+      <c r="M25" s="19" t="n"/>
       <c r="N25" s="19" t="inlineStr"/>
+      <c r="O25" s="19" t="inlineStr"/>
     </row>
     <row r="26" ht="45" customHeight="1">
       <c r="A26" s="17" t="n">
@@ -41714,8 +41848,9 @@
           <t>Passes every gate.</t>
         </is>
       </c>
-      <c r="M26" s="19" t="inlineStr"/>
+      <c r="M26" s="19" t="n"/>
       <c r="N26" s="19" t="inlineStr"/>
+      <c r="O26" s="19" t="inlineStr"/>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="17" t="n">
@@ -41762,8 +41897,9 @@
           <t>Passes every gate.</t>
         </is>
       </c>
-      <c r="M27" s="19" t="inlineStr"/>
+      <c r="M27" s="19" t="n"/>
       <c r="N27" s="19" t="inlineStr"/>
+      <c r="O27" s="19" t="inlineStr"/>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="17" t="n">
@@ -41810,8 +41946,9 @@
           <t>Passes every gate.</t>
         </is>
       </c>
-      <c r="M28" s="19" t="inlineStr"/>
+      <c r="M28" s="19" t="n"/>
       <c r="N28" s="19" t="inlineStr"/>
+      <c r="O28" s="19" t="inlineStr"/>
     </row>
     <row r="29" ht="60" customHeight="1">
       <c r="A29" s="17" t="n">
@@ -41858,12 +41995,13 @@
           <t>Passes every gate.</t>
         </is>
       </c>
-      <c r="M29" s="19" t="inlineStr">
+      <c r="M29" s="19" t="n"/>
+      <c r="N29" s="19" t="inlineStr">
         <is>
           <t>Earnings 2026-08-05</t>
         </is>
       </c>
-      <c r="N29" s="19" t="inlineStr">
+      <c r="O29" s="19" t="inlineStr">
         <is>
           <t>Reports 2026-08-05 (est EPS +2.25). If long &amp; extended, TRIM into the print - do NOT hold full size through a binary. Fresh entry only POST-print if it beats AND holds the gap (PEAD drift = our one measured edge); else awareness-only.</t>
         </is>
@@ -41914,8 +42052,9 @@
           <t>Passes every gate.</t>
         </is>
       </c>
-      <c r="M30" s="19" t="inlineStr"/>
+      <c r="M30" s="19" t="n"/>
       <c r="N30" s="19" t="inlineStr"/>
+      <c r="O30" s="19" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -42011,7 +42150,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N1"/>
+  <autoFilter ref="A1:O1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>

</xml_diff>